<commit_message>
Fix direction_id; minor other fixes
</commit_message>
<xml_diff>
--- a/input-data/NICTD-2026-03-14-for-GTFS.xlsx
+++ b/input-data/NICTD-2026-03-14-for-GTFS.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="67">
   <si>
     <t>NICTD South Shore Line</t>
   </si>
@@ -120,9 +120,6 @@
     <t>Direction</t>
   </si>
   <si>
-    <t>south_shore_WB</t>
-  </si>
-  <si>
     <t>Stop ID</t>
   </si>
   <si>
@@ -205,9 +202,6 @@
   </si>
   <si>
     <t>Extra-0831</t>
-  </si>
-  <si>
-    <t>south_shore_EB</t>
   </si>
   <si>
     <t>Extra-1525</t>
@@ -5856,8 +5850,8 @@
       <c r="A2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="11" t="s">
-        <v>30</v>
+      <c r="B2" s="11">
+        <v>1.0</v>
       </c>
       <c r="C2" s="9"/>
       <c r="D2" s="10"/>
@@ -5919,57 +5913,57 @@
     <row r="3">
       <c r="A3" s="10"/>
       <c r="B3" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="10"/>
       <c r="E3" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="G3" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="H3" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="I3" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="J3" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="K3" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="L3" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="11" t="s">
+      <c r="M3" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="M3" s="11" t="s">
+      <c r="N3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="N3" s="11" t="s">
+      <c r="O3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="O3" s="11" t="s">
+      <c r="P3" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="P3" s="11" t="s">
+      <c r="Q3" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="Q3" s="11" t="s">
+      <c r="R3" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="R3" s="11" t="s">
+      <c r="S3" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="S3" s="11" t="s">
+      <c r="T3" s="11" t="s">
         <v>46</v>
-      </c>
-      <c r="T3" s="11" t="s">
-        <v>47</v>
       </c>
       <c r="U3" s="12"/>
       <c r="V3" s="12"/>
@@ -5981,57 +5975,57 @@
     <row r="4">
       <c r="A4" s="10"/>
       <c r="B4" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="10"/>
       <c r="E4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="T4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="U4" s="9"/>
       <c r="V4" s="9"/>
@@ -6042,16 +6036,16 @@
     </row>
     <row r="5">
       <c r="A5" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="13" t="s">
         <v>52</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>53</v>
       </c>
       <c r="U5" s="10"/>
       <c r="V5" s="10"/>
@@ -6062,16 +6056,16 @@
     </row>
     <row r="6">
       <c r="A6" s="15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>55</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>56</v>
       </c>
       <c r="E6" s="7">
         <v>0.30486111111111114</v>
@@ -6133,16 +6127,16 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B7" s="16" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="15" t="s">
         <v>55</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>56</v>
       </c>
       <c r="E7" s="7">
         <v>0.31180555555555556</v>
@@ -6204,16 +6198,16 @@
     </row>
     <row r="8">
       <c r="A8" s="15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>55</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>56</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7">
@@ -6318,8 +6312,8 @@
       <c r="A2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="11" t="s">
-        <v>59</v>
+      <c r="B2" s="11">
+        <v>0.0</v>
       </c>
       <c r="C2" s="9"/>
       <c r="D2" s="10"/>
@@ -6381,57 +6375,57 @@
     <row r="3">
       <c r="A3" s="10"/>
       <c r="B3" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="10"/>
       <c r="E3" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K3" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N3" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O3" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P3" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q3" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="R3" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S3" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T3" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="U3" s="12"/>
       <c r="V3" s="12"/>
@@ -6443,57 +6437,57 @@
     <row r="4">
       <c r="A4" s="10"/>
       <c r="B4" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="10"/>
       <c r="E4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="T4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="U4" s="9"/>
       <c r="V4" s="9"/>
@@ -6504,16 +6498,16 @@
     </row>
     <row r="5">
       <c r="A5" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="13" t="s">
         <v>52</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>53</v>
       </c>
       <c r="U5" s="10"/>
       <c r="V5" s="10"/>
@@ -6524,13 +6518,13 @@
     </row>
     <row r="6">
       <c r="A6" s="15" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>10</v>
@@ -6598,13 +6592,13 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B7" s="16" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>10</v>
@@ -6672,13 +6666,13 @@
     </row>
     <row r="8">
       <c r="A8" s="15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>10</v>
@@ -6770,7 +6764,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6801,13 +6795,13 @@
     <row r="5">
       <c r="A5" s="5"/>
       <c r="B5" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -7096,7 +7090,7 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -7105,18 +7099,18 @@
     <row r="26">
       <c r="A26" s="5"/>
       <c r="B26" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="18" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -7124,7 +7118,7 @@
     </row>
     <row r="28">
       <c r="A28" s="19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -7132,7 +7126,7 @@
     </row>
     <row r="29">
       <c r="A29" s="18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>

</xml_diff>